<commit_message>
Actualización automática 2026-09-15 16:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0</v>
+        <v>46.44</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>10 de 52</t>
+          <t>11 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -5437,13 +5437,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>21899.88</v>
+        <v>21946.32</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>42590.12</v>
+        <v>42543.68</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3395856721972399</v>
+        <v>0.3403057838424562</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>35361.33</v>
+        <v>35407.77</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>50256.67</v>
+        <v>50210.23</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4130128010465089</v>
+        <v>0.4135552103529632</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-16 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -853,7 +853,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
+        <v>615.6</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>0</v>
@@ -868,7 +868,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>0</v>
+        <v>1491.11</v>
       </c>
       <c r="N6" s="2" t="n">
         <v>0</v>
@@ -901,7 +901,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>0</v>
+        <v>568.71</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>0</v>
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>295.02</v>
+        <v>716.48</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1033,7 +1033,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>853.2</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0</v>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>853.2</v>
+        <v>2098.8</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>0</v>
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0</v>
+        <v>1268.68</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>1 de 52</t>
+          <t>2 de 52</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -3734,14 +3734,14 @@
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
+          <t>6 de 52</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
           <t>4 de 52</t>
         </is>
       </c>
-      <c r="I54" s="4" t="inlineStr">
-        <is>
-          <t>4 de 52</t>
-        </is>
-      </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
           <t>0 de 52</t>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>12 de 52</t>
+          <t>14 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -3950,7 +3950,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>2106.71</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>500</v>
@@ -3977,7 +3977,7 @@
         <v>1082.88</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>295.02</v>
+        <v>1285.19</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>2500</v>
@@ -4031,7 +4031,7 @@
         <v>1089.89</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0</v>
+        <v>853.2</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>1500</v>
@@ -4193,7 +4193,7 @@
         <v>738.72</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>6452.21</v>
+        <v>7697.81</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>5662</v>
@@ -4868,7 +4868,7 @@
         <v>-6.53</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>1268.68</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>4000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>46732.82</v>
+        <v>53197.18</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>
@@ -5173,13 +5173,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1093.89</v>
+        <v>1662.6</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5506.11</v>
+        <v>4937.4</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.1657409090909091</v>
+        <v>0.2519090909090909</v>
       </c>
     </row>
     <row r="4">
@@ -5269,13 +5269,13 @@
         <v>2483</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>3261.6</v>
+        <v>5976</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-778.5999999999999</v>
+        <v>-3493</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.313572291582763</v>
+        <v>2.40676600886025</v>
       </c>
     </row>
     <row r="8">
@@ -5437,13 +5437,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>26132.55</v>
+        <v>29313.8</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>38357.45</v>
+        <v>35176.2</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4052186385486122</v>
+        <v>0.4545479919367343</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>46779.25999999999</v>
+        <v>53243.62</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>38838.73999999999</v>
+        <v>32374.38</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5463717909785325</v>
+        <v>0.6218741386157116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 08:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>874.05</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>433.1</v>
+        <v>2109.16</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -1585,7 +1585,7 @@
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>2870.07</v>
+        <v>7175.17</v>
       </c>
       <c r="M18" s="2" t="n">
         <v>5079.09</v>
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>1207.18</v>
+        <v>3594.16</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -3568,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0</v>
+        <v>830.04</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>14 de 52</t>
+          <t>15 de 52</t>
         </is>
       </c>
       <c r="N54" s="4" t="inlineStr">
@@ -3896,7 +3896,7 @@
         <v>1480.96</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1307.15</v>
+        <v>2983.21</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>3000</v>
@@ -4247,7 +4247,7 @@
         <v>599.59</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>7949.16</v>
+        <v>12254.26</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>5000</v>
@@ -4679,7 +4679,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>3979.78</v>
+        <v>6366.76</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>3000</v>
@@ -5030,7 +5030,7 @@
         <v>406.22</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>830.04</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>1500</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>53434.06</v>
+        <v>62632.24</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>
@@ -5413,13 +5413,13 @@
         <v>2996</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>11862.87</v>
+        <v>16167.97</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-8866.870000000001</v>
+        <v>-13171.97</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>3.959569425901202</v>
+        <v>5.396518691588785</v>
       </c>
     </row>
     <row r="14">
@@ -5437,13 +5437,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>29313.8</v>
+        <v>34206.88</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>35176.2</v>
+        <v>30283.12</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.4545479919367343</v>
+        <v>0.53042146069158</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>53480.5</v>
+        <v>62678.67999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>32137.5</v>
+        <v>22939.32</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6246408465509589</v>
+        <v>0.732073629377</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 16:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -5437,13 +5437,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>33848.62</v>
+        <v>35326.15</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>30641.38</v>
+        <v>29163.85</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.5248661808032253</v>
+        <v>0.5477771747557761</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>62320.42</v>
+        <v>63797.95</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>23297.58</v>
+        <v>21820.05</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.7278892289004648</v>
+        <v>0.745146464528487</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-18 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>993.48</v>
+        <v>2471.01</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -4760,7 +4760,7 @@
         <v>13198.82</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>993.48</v>
+        <v>2471.01</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>2000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>62273.98</v>
+        <v>63751.51</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 14:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>-358.26</v>
+        <v>-330.88</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -4139,7 +4139,7 @@
         <v>3184.27</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>-121.38</v>
+        <v>-94</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2000</v>
@@ -5074,7 +5074,7 @@
         <v>51483.74</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>70848.91</v>
+        <v>70876.28999999999</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>76987</v>
@@ -5437,13 +5437,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>38646</v>
+        <v>38673.38</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>25844</v>
+        <v>25816.62</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.5992556985579159</v>
+        <v>0.5996802605055047</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5480,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>72129.63</v>
+        <v>72157.00999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>13488.37</v>
+        <v>13460.99</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8424587119530941</v>
+        <v>0.8427785045200775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 16:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CEDEÑO MACIAS FRANCISCO ARMANDO</t>
+          <t>CARANGUI ARMIJOS LUIS FRANCISCO</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>3085.71</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -1374,14 +1374,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CERAMIKASA S.A.S.</t>
+          <t>CEDEÑO MACIAS FRANCISCO ARMANDO</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1093.89</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>2098.8</v>
+        <v>0</v>
       </c>
       <c r="I15" s="2" t="n">
         <v>0</v>
@@ -1402,13 +1402,13 @@
         <v>0</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>118.44</v>
+        <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>4511.44</v>
+        <v>0</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1434,14 +1434,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CONSORCIO MUELLE CENTRO DE ARTE</t>
+          <t>CERAMIKASA S.A.S.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>1093.89</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>0</v>
+        <v>2098.8</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>0</v>
@@ -1462,13 +1462,13 @@
         <v>0</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>118.44</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>4511.44</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DECOGARCIA S.A.S.</t>
+          <t>CONSORCIO MUELLE CENTRO DE ARTE</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DECORPISOS CIA. LTDA</t>
+          <t>DECOGARCIA S.A.S.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1585,10 +1585,10 @@
         <v>0</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>7175.17</v>
+        <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>5079.09</v>
+        <v>0</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ENCARNACION ERAS KATTY ELIZABETH</t>
+          <t>DECORPISOS CIA. LTDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1645,10 +1645,10 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>9522.85</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>5079.09</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FADESE C LTDA</t>
+          <t>ENCARNACION ERAS KATTY ELIZABETH</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FAREZ ARCINIEGA DIANA FRANCISCA</t>
+          <t>FADESE C LTDA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1753,7 +1753,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>142.2</v>
+        <v>0</v>
       </c>
       <c r="I21" s="2" t="n">
         <v>0</v>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FEIJOO FEIJOO CRISTOPHER ANDRE</t>
+          <t>FAREZ ARCINIEGA DIANA FRANCISCA</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1813,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>0</v>
+        <v>142.2</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
@@ -1854,11 +1854,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FEIJOO MARIN MAURICIO ENRIQUE</t>
+          <t>FEIJOO FEIJOO CRISTOPHER ANDRE</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>118.96</v>
+        <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>0</v>
@@ -1885,10 +1885,10 @@
         <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>2178.91</v>
+        <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>4745.63</v>
+        <v>0</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -1914,11 +1914,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GARCIA YEPEZ MARIA ISABEL</t>
+          <t>FEIJOO MARIN MAURICIO ENRIQUE</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>0</v>
@@ -1945,10 +1945,10 @@
         <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0</v>
+        <v>2178.91</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>4745.63</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ILLINGWORTH VILLA ALLAN FRANCISCO</t>
+          <t>GARCIA YEPEZ MARIA ISABEL</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IMPORT NOVUM MADE S.A.S.</t>
+          <t>ILLINGWORTH VILLA ALLAN FRANCISCO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LATACELA ZUÑIGA JUAN FERNANDO</t>
+          <t>IMPORT NOVUM MADE S.A.S.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2128,7 +2128,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>17.2</v>
+        <v>0</v>
       </c>
       <c r="N27" s="2" t="n">
         <v>0</v>
@@ -2154,7 +2154,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MADECOR-HOME CENTER S.A.S.</t>
+          <t>LATACELA ZUÑIGA JUAN FERNANDO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2176,7 +2176,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>45.53</v>
+        <v>0</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0</v>
@@ -2185,10 +2185,10 @@
         <v>0</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>1052.57</v>
+        <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>2481.21</v>
+        <v>17.2</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MARQUEZ CELI ALFREDO NICANOR</t>
+          <t>MADECOR-HOME CENTER S.A.S.</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2236,7 +2236,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>45.53</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0</v>
@@ -2245,10 +2245,10 @@
         <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>1052.57</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>3921.21</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
+          <t>MARQUEZ CELI ALFREDO NICANOR</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2305,7 +2305,7 @@
         <v>0</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>977.16</v>
+        <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>0</v>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MEGAUNIMAC CIA.LTDA.</t>
+          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>0</v>
+        <v>977.16</v>
       </c>
       <c r="M31" s="2" t="n">
         <v>0</v>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>OCHOA CUEVA LUIS DAVID</t>
+          <t>MEGAUNIMAC CIA.LTDA.</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
+          <t>OCHOA CUEVA LUIS DAVID</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2545,10 +2545,10 @@
         <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>1990.28</v>
+        <v>0</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>3323.05</v>
+        <v>0</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2593,10 +2593,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>853.2</v>
+        <v>0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>574.27</v>
+        <v>0</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0</v>
@@ -2605,10 +2605,10 @@
         <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>0</v>
+        <v>1990.28</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>3594.16</v>
+        <v>3323.05</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2653,10 +2653,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>0</v>
+        <v>853.2</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>0</v>
+        <v>574.27</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>3594.16</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>2928.27</v>
+        <v>0</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>2928.27</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2893,10 +2893,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>1242</v>
+        <v>0</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>267.62</v>
+        <v>0</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0</v>
@@ -2905,10 +2905,10 @@
         <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>761.87</v>
+        <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>40.02</v>
+        <v>0</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -2934,7 +2934,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2953,10 +2953,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>0</v>
+        <v>1242</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0</v>
+        <v>267.62</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0</v>
@@ -2965,10 +2965,10 @@
         <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>0</v>
+        <v>761.87</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>0</v>
+        <v>114.63</v>
       </c>
       <c r="N41" s="2" t="n">
         <v>0</v>
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
+          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3148,7 +3148,7 @@
         <v>0</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>1268.68</v>
+        <v>0</v>
       </c>
       <c r="N44" s="2" t="n">
         <v>0</v>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3208,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>1362.16</v>
+        <v>1268.68</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>0</v>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0</v>
+        <v>1362.16</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3388,7 +3388,7 @@
         <v>0</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>219.81</v>
+        <v>0</v>
       </c>
       <c r="N48" s="2" t="n">
         <v>0</v>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3448,7 +3448,7 @@
         <v>0</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0</v>
+        <v>219.81</v>
       </c>
       <c r="N49" s="2" t="n">
         <v>0</v>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3568,7 +3568,7 @@
         <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>830.04</v>
+        <v>0</v>
       </c>
       <c r="N51" s="2" t="n">
         <v>0</v>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3628,7 +3628,7 @@
         <v>0</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>1280.72</v>
+        <v>830.04</v>
       </c>
       <c r="N52" s="2" t="n">
         <v>0</v>
@@ -3654,137 +3654,197 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="2" t="n">
+        <v>1280.72</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
-      <c r="C53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q53" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R53" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>2 de 52</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>3 de 52</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>7 de 52</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
-        <is>
-          <t>4 de 52</t>
-        </is>
-      </c>
-      <c r="J54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="K54" s="4" t="inlineStr">
-        <is>
-          <t>2 de 52</t>
-        </is>
-      </c>
-      <c r="L54" s="4" t="inlineStr">
-        <is>
-          <t>10 de 52</t>
-        </is>
-      </c>
-      <c r="M54" s="4" t="inlineStr">
-        <is>
-          <t>18 de 52</t>
-        </is>
-      </c>
-      <c r="N54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="O54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="P54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="Q54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
-        </is>
-      </c>
-      <c r="R54" s="4" t="inlineStr">
-        <is>
-          <t>0 de 52</t>
+      <c r="C54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>2 de 53</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>3 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>7 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>4 de 53</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>2 de 53</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>10 de 53</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>19 de 53</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="R55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4153,7 +4213,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CEDEÑO MACIAS FRANCISCO ARMANDO</t>
+          <t>CARANGUI ARMIJOS LUIS FRANCISCO</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -4163,13 +4223,13 @@
         <v>0</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>676.8</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>3085.71</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4180,23 +4240,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CERAMIKASA S.A.S.</t>
+          <t>CEDEÑO MACIAS FRANCISCO ARMANDO</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2910.78</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13338.07</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>738.72</v>
+        <v>676.8</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>7822.57</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>5662</v>
+        <v>500</v>
       </c>
     </row>
     <row r="15">
@@ -4207,23 +4267,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DECOGARCIA S.A.S.</t>
+          <t>CERAMIKASA S.A.S.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-589.36</v>
+        <v>2910.78</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1355.61</v>
+        <v>13338.07</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>210.12</v>
+        <v>738.72</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>7822.57</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0</v>
+        <v>5662</v>
       </c>
     </row>
     <row r="16">
@@ -4234,23 +4294,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DECORPISOS CIA. LTDA</t>
+          <t>DECOGARCIA S.A.S.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>16.74</v>
+        <v>-589.36</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5644.57</v>
+        <v>1355.61</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>599.59</v>
+        <v>210.12</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>12254.26</v>
+        <v>0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -4261,23 +4321,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ENCARNACION ERAS KATTY ELIZABETH</t>
+          <t>DECORPISOS CIA. LTDA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1772.67</v>
+        <v>16.74</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>74.61</v>
+        <v>5644.57</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0</v>
+        <v>599.59</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>14601.94</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="18">
@@ -4288,14 +4348,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FADESE C LTDA</t>
+          <t>ENCARNACION ERAS KATTY ELIZABETH</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0</v>
+        <v>1772.67</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0</v>
+        <v>74.61</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -4304,7 +4364,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
@@ -4315,7 +4375,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FAREZ ARCINIEGA DIANA FRANCISCA</t>
+          <t>FADESE C LTDA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -4328,7 +4388,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>142.2</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>0</v>
@@ -4342,7 +4402,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FEIJOO FEIJOO CRISTOPHER ANDRE</t>
+          <t>FAREZ ARCINIEGA DIANA FRANCISCA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -4355,10 +4415,10 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>142.2</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -4369,23 +4429,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FEIJOO MARIN MAURICIO ENRIQUE</t>
+          <t>FEIJOO FEIJOO CRISTOPHER ANDRE</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>4640.2</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>3662.98</v>
+        <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>7043.5</v>
+        <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>4651</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="22">
@@ -4396,23 +4456,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GARCIA YEPEZ MARIA ISABEL</t>
+          <t>FEIJOO MARIN MAURICIO ENRIQUE</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>4640.2</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0</v>
+        <v>3662.98</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>7043.5</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>4651</v>
       </c>
     </row>
     <row r="23">
@@ -4423,7 +4483,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ILLINGWORTH VILLA ALLAN FRANCISCO</t>
+          <t>GARCIA YEPEZ MARIA ISABEL</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -4439,7 +4499,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -4450,7 +4510,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IMPORT NOVUM MADE S.A.S.</t>
+          <t>ILLINGWORTH VILLA ALLAN FRANCISCO</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -4466,7 +4526,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25">
@@ -4477,23 +4537,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LATACELA ZUÑIGA JUAN FERNANDO</t>
+          <t>IMPORT NOVUM MADE S.A.S.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>-65.18000000000001</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>1415.23</v>
+        <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>17.2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -4504,20 +4564,20 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MADECOR-HOME CENTER S.A.S.</t>
+          <t>LATACELA ZUÑIGA JUAN FERNANDO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2107.43</v>
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>3862.86</v>
+        <v>-65.18000000000001</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1914.76</v>
+        <v>1415.23</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>3579.31</v>
+        <v>17.2</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3000</v>
@@ -4531,23 +4591,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MARQUEZ CELI ALFREDO NICANOR</t>
+          <t>MADECOR-HOME CENTER S.A.S.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>0</v>
+        <v>2107.43</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0</v>
+        <v>3862.86</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>1914.76</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>5019.31</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="28">
@@ -4558,23 +4618,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
+          <t>MARQUEZ CELI ALFREDO NICANOR</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>16.74</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>179.92</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>1030.52</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>977.16</v>
+        <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -4585,20 +4645,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MEGAUNIMAC CIA.LTDA.</t>
+          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1656.06</v>
+        <v>16.74</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0</v>
+        <v>179.92</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>3161.5</v>
+        <v>1030.52</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0</v>
+        <v>977.16</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>3000</v>
@@ -4612,23 +4672,23 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
+          <t>MEGAUNIMAC CIA.LTDA.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>306.5</v>
+        <v>1656.06</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>36.2</v>
+        <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>3161.5</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="31">
@@ -4639,23 +4699,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>164.48</v>
+        <v>306.5</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>12800.81</v>
+        <v>36.2</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>11244.69</v>
+        <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>5429.33</v>
+        <v>0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>9000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="32">
@@ -4666,23 +4726,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>3107.31</v>
+        <v>164.48</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>836.66</v>
+        <v>12800.81</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0</v>
+        <v>11244.69</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>6366.76</v>
+        <v>5429.33</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>3000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="33">
@@ -4693,23 +4753,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1714.5</v>
+        <v>3107.31</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>836.66</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>7260.45</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="34">
@@ -4720,14 +4780,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0</v>
+        <v>1714.5</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>36.29</v>
+        <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>0</v>
@@ -4736,7 +4796,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35">
@@ -4747,23 +4807,23 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>118.96</v>
+        <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>104.73</v>
+        <v>36.29</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>13198.82</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>2928.27</v>
+        <v>0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -4774,23 +4834,23 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>669.0599999999999</v>
+        <v>118.96</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>1465.48</v>
+        <v>104.73</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
+        <v>13198.82</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>2928.27</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="37">
@@ -4801,23 +4861,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>0</v>
+        <v>669.0599999999999</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>1388.57</v>
+        <v>1465.48</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>3984.02</v>
+        <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>3462.99</v>
+        <v>0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="38">
@@ -4828,23 +4888,23 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>0</v>
+        <v>1388.57</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0</v>
+        <v>3984.02</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>3537.6</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="39">
@@ -4855,23 +4915,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>8325.82</v>
+        <v>0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>-6.53</v>
+        <v>0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>1268.68</v>
+        <v>0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -4882,23 +4942,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>90.98</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>203.94</v>
+        <v>8325.82</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0</v>
+        <v>-6.53</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>1362.16</v>
+        <v>1268.68</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="41">
@@ -4909,23 +4969,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>118.96</v>
+        <v>90.98</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>1819.81</v>
+        <v>203.94</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>1362.16</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="42">
@@ -4936,14 +4996,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>0</v>
+        <v>118.96</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>0</v>
+        <v>1819.81</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>0</v>
@@ -4952,7 +5012,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="43">
@@ -4963,7 +5023,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -4976,7 +5036,7 @@
         <v>0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>219.81</v>
+        <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>0</v>
@@ -4990,20 +5050,20 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>-143.32</v>
+        <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0</v>
+        <v>219.81</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>0</v>
@@ -5017,23 +5077,23 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>0</v>
+        <v>-143.32</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>406.22</v>
+        <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>837.78</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -5044,39 +5104,66 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>406.22</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>837.78</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="C47" s="5" t="n">
+      <c r="C47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="5" t="n">
         <v>21100.38</v>
       </c>
-      <c r="D47" s="5" t="n">
+      <c r="D48" s="5" t="n">
         <v>85092.72</v>
       </c>
-      <c r="E47" s="5" t="n">
+      <c r="E48" s="5" t="n">
         <v>51483.74</v>
       </c>
-      <c r="F47" s="5" t="n">
-        <v>70876.28999999999</v>
-      </c>
-      <c r="G47" s="5" t="n">
+      <c r="F48" s="5" t="n">
+        <v>78717.98</v>
+      </c>
+      <c r="G48" s="5" t="n">
         <v>76987</v>
       </c>
     </row>
@@ -5197,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2512.09</v>
+        <v>3405.78</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3019.91</v>
+        <v>2126.22</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.4541015907447578</v>
+        <v>0.615650759219089</v>
       </c>
     </row>
     <row r="5">
@@ -5413,13 +5500,13 @@
         <v>2996</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20524.67</v>
+        <v>22872.35</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-17528.67</v>
+        <v>-19876.35</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>6.850690921228304</v>
+        <v>7.634295727636848</v>
       </c>
     </row>
     <row r="14">
@@ -5437,13 +5524,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>38673.38</v>
+        <v>43273.7</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>25816.62</v>
+        <v>21216.3</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.5996802605055047</v>
+        <v>0.6710141107148395</v>
       </c>
     </row>
     <row r="15">
@@ -5480,13 +5567,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>72157.00999999999</v>
+        <v>79998.7</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>13460.99</v>
+        <v>5619.299999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.8427785045200775</v>
+        <v>0.9343677731318181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 15:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>1362.16</v>
+        <v>1374.06</v>
       </c>
       <c r="N46" s="2" t="n">
         <v>0</v>
@@ -4982,7 +4982,7 @@
         <v>0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>1362.16</v>
+        <v>1374.06</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>1500</v>
@@ -5161,7 +5161,7 @@
         <v>51483.74</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>78717.98</v>
+        <v>78729.88</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5524,13 +5524,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>43273.7</v>
+        <v>43285.6</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>21216.3</v>
+        <v>21204.4</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6710141107148395</v>
+        <v>0.6711986354473561</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>79998.7</v>
+        <v>80010.60000000001</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>5619.299999999999</v>
+        <v>5607.400000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.9343677731318181</v>
+        <v>0.9345067625966503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 14:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -3601,7 +3601,7 @@
         <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>0</v>
+        <v>92.08</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>3 de 53</t>
+          <t>4 de 53</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
@@ -5117,7 +5117,7 @@
         <v>406.22</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>837.78</v>
+        <v>929.86</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>1500</v>
@@ -5161,7 +5161,7 @@
         <v>51483.74</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>78537.02</v>
+        <v>78629.10000000001</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5260,13 +5260,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1999.79</v>
+        <v>2091.87</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4600.21</v>
+        <v>4508.13</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.3029984848484849</v>
+        <v>0.31695</v>
       </c>
     </row>
     <row r="4">
@@ -5567,13 +5567,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>79817.73999999999</v>
+        <v>79909.81999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>5800.260000000002</v>
+        <v>5708.180000000002</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.9322541988834122</v>
+        <v>0.9333296736667522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>874.05</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>2109.16</v>
+        <v>2177.39</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>4231.94</v>
+        <v>5092.94</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>3006.03</v>
@@ -1621,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>649.96</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1813,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>142.2</v>
+        <v>284.4</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
@@ -2248,7 +2248,7 @@
         <v>1052.57</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>3921.21</v>
+        <v>4538.35</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2542,7 +2542,7 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>61.92</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0</v>
+        <v>1324.3</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -3774,42 +3774,42 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
+          <t>5 de 53</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>0 de 53</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>7 de 53</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
           <t>4 de 53</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>0 de 53</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>7 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>4 de 53</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>19 de 53</t>
+          <t>20 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>1480.96</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2983.21</v>
+        <v>3051.44</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>3000</v>
@@ -3983,7 +3983,7 @@
         <v>-373.57</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>7237.97</v>
+        <v>8098.97</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>6174</v>
@@ -4334,7 +4334,7 @@
         <v>599.59</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>14601.94</v>
+        <v>15251.9</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>5000</v>
@@ -4415,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>142.2</v>
+        <v>284.4</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>0</v>
@@ -4604,7 +4604,7 @@
         <v>1914.76</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>5019.31</v>
+        <v>5636.45</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>3000</v>
@@ -4712,7 +4712,7 @@
         <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>61.92</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>500</v>
@@ -4739,7 +4739,7 @@
         <v>11244.69</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>5429.33</v>
+        <v>5568.53</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>9000</v>
@@ -4874,7 +4874,7 @@
         <v>0</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>1324.3</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>1500</v>
@@ -5161,7 +5161,7 @@
         <v>51483.74</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>78629.10000000001</v>
+        <v>82493.05</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5260,13 +5260,13 @@
         <v>6600</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2091.87</v>
+        <v>2741.83</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4508.13</v>
+        <v>3858.17</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.31695</v>
+        <v>0.4154287878787878</v>
       </c>
     </row>
     <row r="4">
@@ -5356,13 +5356,13 @@
         <v>2483</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>6118.2</v>
+        <v>6260.4</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-3635.2</v>
+        <v>-3777.4</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2.464035440998792</v>
+        <v>2.521304873137334</v>
       </c>
     </row>
     <row r="8">
@@ -5452,13 +5452,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>355.32</v>
+        <v>417.24</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>372.68</v>
+        <v>310.76</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.4880769230769231</v>
+        <v>0.5731318681318681</v>
       </c>
     </row>
     <row r="12">
@@ -5476,13 +5476,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>116</v>
+        <v>255.2</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>234</v>
+        <v>94.80000000000001</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.3314285714285714</v>
+        <v>0.7291428571428571</v>
       </c>
     </row>
     <row r="13">
@@ -5500,13 +5500,13 @@
         <v>2996</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>22872.35</v>
+        <v>23733.35</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-19876.35</v>
+        <v>-20737.35</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>7.634295727636848</v>
+        <v>7.921678905206942</v>
       </c>
     </row>
     <row r="14">
@@ -5524,13 +5524,13 @@
         <v>64490</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>43166.92</v>
+        <v>45176.59</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>21323.08</v>
+        <v>19313.41</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6693583501318033</v>
+        <v>0.7005208559466584</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>85618</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>79909.81999999999</v>
+        <v>83773.76999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>5708.180000000002</v>
+        <v>1844.230000000003</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.9333296736667522</v>
+        <v>0.9784597864934942</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-01 16:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>1554.19</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>1 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4739,7 +4739,7 @@
         <v>5568.53</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>0</v>
+        <v>1554.19</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>9000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0</v>
+        <v>1554.19</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-01 17:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -483,7 +483,7 @@
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
@@ -3559,7 +3559,7 @@
         <v>0</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0</v>
+        <v>218.16</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>1 de 53</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
@@ -5090,7 +5090,7 @@
         <v>0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0</v>
+        <v>218.16</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1554.19</v>
+        <v>1772.35</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-02 08:30:14
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>2064.1</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>1 de 53</t>
+          <t>2 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4307,7 +4307,7 @@
         <v>-40.75</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>2064.1</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>1772.35</v>
+        <v>3836.45</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-05 15:30:14
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>0</v>
+        <v>2872.22</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4847,7 +4847,7 @@
         <v>2928.27</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>0</v>
+        <v>2872.22</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>2000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>3889.89</v>
+        <v>6762.11</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 17:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1402,7 +1402,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0</v>
+        <v>1184.4</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>0</v>
+        <v>130.64</v>
       </c>
       <c r="M31" s="2" t="n">
         <v>0</v>
@@ -3809,12 +3809,12 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>1 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>0 de 53</t>
+          <t>1 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
@@ -4172,7 +4172,7 @@
         <v>1341.02</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>5156.2</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>2500</v>
@@ -4253,7 +4253,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0</v>
+        <v>2018.88</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>500</v>
@@ -4658,7 +4658,7 @@
         <v>914.71</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0</v>
+        <v>130.64</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>3000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>11079.22</v>
+        <v>18384.94</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 08:30:14
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -805,7 +805,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>1156.78</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -1645,7 +1645,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>0</v>
+        <v>391.91</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>1851.43</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>208.66</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>253.44</v>
@@ -2602,7 +2602,7 @@
         <v>0</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>78.95999999999999</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -3809,17 +3809,17 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>1 de 53</t>
+          <t>2 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>1 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>5 de 53</t>
+          <t>6 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
         <v>11995.13</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>1156.78</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>6174</v>
@@ -4334,7 +4334,7 @@
         <v>16486.18</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1851.43</v>
+        <v>2243.34</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>5000</v>
@@ -4604,7 +4604,7 @@
         <v>5754.95</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>284.84</v>
+        <v>493.5</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>3000</v>
@@ -4739,7 +4739,7 @@
         <v>5568.53</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1530.64</v>
+        <v>2043.12</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>9000</v>
@@ -4766,7 +4766,7 @@
         <v>7260.45</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0</v>
+        <v>489.18</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>3000</v>
@@ -4901,7 +4901,7 @@
         <v>3463.42</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0</v>
+        <v>466.14</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>2000</v>
@@ -4955,7 +4955,7 @@
         <v>1268.68</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0</v>
+        <v>512.22</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>4000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>18403.64</v>
+        <v>22141.01</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>5847.35</v>
+        <v>5911.65</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4199,7 +4199,7 @@
         <v>-94</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>2731.67</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2000</v>
@@ -4847,7 +4847,7 @@
         <v>2928.27</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>5847.35</v>
+        <v>5911.65</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>2000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>25097.44</v>
+        <v>27893.41</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5186,7 +5186,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>53.44</v>
+        <v>2428.28</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5478.56</v>
+        <v>3103.72</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.009660159074475778</v>
+        <v>0.4389515545914678</v>
       </c>
     </row>
     <row r="5">
@@ -5476,13 +5476,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>7891.74</v>
+        <v>8248.57</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>-7541.74</v>
+        <v>-7898.57</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>22.54782857142857</v>
+        <v>23.56734285714286</v>
       </c>
     </row>
     <row r="13">
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13442.77</v>
+        <v>13507.07</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>59245.23999999999</v>
+        <v>59180.94</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1849379285524532</v>
+        <v>0.1858225311162047</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>25097.44</v>
+        <v>27893.41</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>65042.56999999999</v>
+        <v>62246.6</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2784273043679494</v>
+        <v>0.3094453839088769</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-14 17:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>887.4400000000001</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -802,7 +802,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>0</v>
+        <v>71.06</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>1156.78</v>
@@ -2248,7 +2248,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>208.66</v>
+        <v>293.57</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>253.44</v>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>6 de 53</t>
+          <t>7 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -3956,7 +3956,7 @@
         <v>3051.44</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>887.4400000000001</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>3000</v>
@@ -3983,7 +3983,7 @@
         <v>11995.13</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1156.78</v>
+        <v>1227.84</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>6174</v>
@@ -4604,7 +4604,7 @@
         <v>5754.95</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>493.5</v>
+        <v>5346.9</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>3000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>27893.41</v>
+        <v>33705.31</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2428.28</v>
+        <v>7196.77</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3103.72</v>
+        <v>-1664.77</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.4389515545914678</v>
+        <v>1.300934562545192</v>
       </c>
     </row>
     <row r="5">
@@ -5452,13 +5452,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1263.36</v>
+        <v>1334.42</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-535.3599999999999</v>
+        <v>-606.4200000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.735384615384615</v>
+        <v>1.832994505494506</v>
       </c>
     </row>
     <row r="12">
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13507.07</v>
+        <v>14479.42</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>59180.94</v>
+        <v>58208.59</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1858225311162047</v>
+        <v>0.1991995653753625</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>27893.41</v>
+        <v>33705.31</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>62246.6</v>
+        <v>56434.7</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3094453839088769</v>
+        <v>0.3739217468469329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 14:30:15
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2608,7 +2608,7 @@
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>1530.64</v>
+        <v>1536.22</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -4739,7 +4739,7 @@
         <v>5568.53</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>2043.12</v>
+        <v>2048.7</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>9000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>33738.71</v>
+        <v>33744.29</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>14496.16</v>
+        <v>14501.74</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>58191.84999999999</v>
+        <v>58186.27</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1994298647053345</v>
+        <v>0.1995066311486585</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>33738.71000000001</v>
+        <v>33744.29</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>56401.29999999999</v>
+        <v>56395.71999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3742922815295894</v>
+        <v>0.3743541852280691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 08:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>25.93</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -1708,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>25.93</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>8 de 53</t>
+          <t>10 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4226,7 +4226,7 @@
         <v>3085.71</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0</v>
+        <v>42.59</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -4361,7 +4361,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>42.59</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>500</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>33744.29</v>
+        <v>33829.47</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5184,7 +5184,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7213.43</v>
+        <v>7246.75</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-1681.43</v>
+        <v>-1714.75</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1.303946131597975</v>
+        <v>1.309969269703543</v>
       </c>
     </row>
     <row r="5">
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>14501.74</v>
+        <v>14553.6</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>58186.27</v>
+        <v>58134.41</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1995066311486585</v>
+        <v>0.2002200913190497</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>33744.29</v>
+        <v>33829.47</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>56395.71999999999</v>
+        <v>56310.54</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3743541852280691</v>
+        <v>0.3752991596073708</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 10:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>5911.65</v>
+        <v>5955.02</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4847,7 +4847,7 @@
         <v>2928.27</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>5911.65</v>
+        <v>5955.02</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>2000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>33829.47</v>
+        <v>33872.84</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5184,7 +5184,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>14553.6</v>
+        <v>14596.97</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>58134.41</v>
+        <v>58091.03999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2002200913190497</v>
+        <v>0.2008167509332007</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>33829.47</v>
+        <v>33872.84</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>56310.54</v>
+        <v>56267.16999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3752991596073708</v>
+        <v>0.3757803000021855</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 15:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R55"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MADECOR-HOME CENTER S.A.S.</t>
+          <t>LISLOP S.A</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>299.15</v>
+        <v>25.42</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>253.44</v>
+        <v>0</v>
       </c>
       <c r="O29" s="2" t="n">
         <v>0</v>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MARQUEZ CELI ALFREDO NICANOR</t>
+          <t>MADECOR-HOME CENTER S.A.S.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2308,10 +2308,10 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0</v>
+        <v>299.15</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0</v>
+        <v>253.44</v>
       </c>
       <c r="O30" s="2" t="n">
         <v>0</v>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
+          <t>MARQUEZ CELI ALFREDO NICANOR</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2365,7 +2365,7 @@
         <v>0</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>130.64</v>
+        <v>0</v>
       </c>
       <c r="M31" s="2" t="n">
         <v>0</v>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MEGAUNIMAC CIA.LTDA.</t>
+          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2425,7 +2425,7 @@
         <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>0</v>
+        <v>130.64</v>
       </c>
       <c r="M32" s="2" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OCHOA CUEVA LUIS DAVID</t>
+          <t>MEGAUNIMAC CIA.LTDA.</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
+          <t>OCHOA CUEVA LUIS DAVID</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2602,13 +2602,13 @@
         <v>0</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>78.95999999999999</v>
+        <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>1536.22</v>
+        <v>0</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2662,13 +2662,13 @@
         <v>0</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>0</v>
+        <v>78.95999999999999</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>0</v>
+        <v>1536.22</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>5955.02</v>
+        <v>0</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2908,7 +2908,7 @@
         <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>0</v>
+        <v>5955.02</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>0</v>
@@ -2934,7 +2934,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
+          <t>QUINCHE ALCIVAR ARGENTINA DEL ROCIO</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>RAMIREZ APOLO JOBANI DE JESUS</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -3294,7 +3294,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -3414,7 +3414,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SANDIEGO NEUMATICOS &amp; SERVICIOS CIA LTDA</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -3559,7 +3559,7 @@
         <v>0</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>218.16</v>
+        <v>0</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -3619,7 +3619,7 @@
         <v>0</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0</v>
+        <v>218.16</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -3714,137 +3714,197 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
+          <t>WONG SANCHEZ CLAUDIA PAULINA</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>ZUÑIGA CORONEL MARCIA LUZMILA</t>
         </is>
       </c>
-      <c r="C54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="K55" s="4" t="inlineStr">
-        <is>
-          <t>3 de 53</t>
-        </is>
-      </c>
-      <c r="L55" s="4" t="inlineStr">
-        <is>
-          <t>3 de 53</t>
-        </is>
-      </c>
-      <c r="M55" s="4" t="inlineStr">
-        <is>
-          <t>10 de 53</t>
-        </is>
-      </c>
-      <c r="N55" s="4" t="inlineStr">
-        <is>
-          <t>1 de 53</t>
-        </is>
-      </c>
-      <c r="O55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="P55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="Q55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
-        </is>
-      </c>
-      <c r="R55" s="4" t="inlineStr">
-        <is>
-          <t>0 de 53</t>
+      <c r="C55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>3 de 54</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>11 de 54</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>1 de 54</t>
+        </is>
+      </c>
+      <c r="O56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="P56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="Q56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
+        </is>
+      </c>
+      <c r="R56" s="4" t="inlineStr">
+        <is>
+          <t>0 de 54</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4591,23 +4651,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MADECOR-HOME CENTER S.A.S.</t>
+          <t>LISLOP S.A</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>3862.86</v>
+        <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1914.76</v>
+        <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>5754.95</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>5352.48</v>
+        <v>25.42</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -4618,23 +4678,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MARQUEZ CELI ALFREDO NICANOR</t>
+          <t>MADECOR-HOME CENTER S.A.S.</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>0</v>
+        <v>3862.86</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0</v>
+        <v>1914.76</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0</v>
+        <v>5754.95</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0</v>
+        <v>5352.48</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="29">
@@ -4645,23 +4705,23 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
+          <t>MARQUEZ CELI ALFREDO NICANOR</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>179.92</v>
+        <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1030.52</v>
+        <v>0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>914.71</v>
+        <v>0</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>130.64</v>
+        <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -4672,20 +4732,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MEGAUNIMAC CIA.LTDA.</t>
+          <t>MATUTE GUANOLIQUE DOLORES MATILDE</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0</v>
+        <v>179.92</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3161.5</v>
+        <v>1030.52</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>914.71</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>130.64</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>3000</v>
@@ -4699,23 +4759,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
+          <t>MEGAUNIMAC CIA.LTDA.</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>36.2</v>
+        <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>3161.5</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>61.92</v>
+        <v>0</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="32">
@@ -4726,23 +4786,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN KLEBER ERWIN</t>
+          <t>OJEDA GONZALEZ EDWIN FERNANDO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>12800.81</v>
+        <v>36.2</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>11244.69</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>5568.53</v>
+        <v>61.92</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>2048.7</v>
+        <v>0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>9000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="33">
@@ -4753,23 +4813,23 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ORTEGA ROMAN LUIS FERNANDO</t>
+          <t>ORTEGA ROMAN KLEBER ERWIN</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>836.66</v>
+        <v>12800.81</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0</v>
+        <v>11244.69</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>7260.45</v>
+        <v>5568.53</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>489.18</v>
+        <v>2048.7</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>3000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="34">
@@ -4780,23 +4840,23 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA DORIS PRICILA</t>
+          <t>ORTEGA ROMAN LUIS FERNANDO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0</v>
+        <v>836.66</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0</v>
+        <v>7260.45</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>489.18</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="35">
@@ -4807,11 +4867,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
+          <t>PACHECO NIVICELA DORIS PRICILA</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>36.29</v>
+        <v>0</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>0</v>
@@ -4823,7 +4883,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="36">
@@ -4834,23 +4894,23 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PEREZ ROSALES EDGAR RICARDO</t>
+          <t>PACHECO NIVICELA SANDRA ELISABETH</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>104.73</v>
+        <v>36.29</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>13198.82</v>
+        <v>0</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>2928.27</v>
+        <v>0</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>5955.02</v>
+        <v>0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -4861,23 +4921,23 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
+          <t>PEREZ ROSALES EDGAR RICARDO</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1465.48</v>
+        <v>104.73</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0</v>
+        <v>13198.82</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1324.3</v>
+        <v>2928.27</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0</v>
+        <v>5955.02</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="38">
@@ -4888,23 +4948,23 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>QUEZADA VEGA JAIME PATRICIO</t>
+          <t>PEÑALOZA LOPEZ RONALD STALIN</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>1388.57</v>
+        <v>1465.48</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>3984.02</v>
+        <v>0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>3463.42</v>
+        <v>1324.3</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>466.14</v>
+        <v>0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="39">
@@ -4915,23 +4975,23 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REYES MOSCOSO NARCISA DE JESUS</t>
+          <t>QUEZADA VEGA JAIME PATRICIO</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>0</v>
+        <v>1388.57</v>
       </c>
       <c r="D39" s="2" t="n">
-        <v>0</v>
+        <v>3984.02</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0</v>
+        <v>3463.42</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0</v>
+        <v>466.14</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="40">
@@ -4942,23 +5002,23 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROJAS SANCHEZ LADY MARGOT</t>
+          <t>REYES MOSCOSO NARCISA DE JESUS</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>8325.82</v>
+        <v>0</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>-6.53</v>
+        <v>0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>1268.68</v>
+        <v>0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>512.22</v>
+        <v>0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -4969,23 +5029,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROMERO RODAS SILVIA MARELIS</t>
+          <t>ROJAS SANCHEZ LADY MARGOT</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>203.94</v>
+        <v>8325.82</v>
       </c>
       <c r="D41" s="2" t="n">
-        <v>0</v>
+        <v>-6.53</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1374.06</v>
+        <v>1268.68</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>0</v>
+        <v>512.22</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="42">
@@ -4996,23 +5056,23 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
+          <t>ROMERO RODAS SILVIA MARELIS</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>1819.81</v>
+        <v>203.94</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0</v>
+        <v>1374.06</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="43">
@@ -5023,11 +5083,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SALAS NOBLECILLA MARIA SUSANA</t>
+          <t>RUIZ TINIZARAY YOHANNA MARYURI</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>0</v>
+        <v>1819.81</v>
       </c>
       <c r="D43" s="2" t="n">
         <v>0</v>
@@ -5039,7 +5099,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="44">
@@ -5050,7 +5110,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
+          <t>SALAS NOBLECILLA MARIA SUSANA</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -5060,7 +5120,7 @@
         <v>0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>219.81</v>
+        <v>0</v>
       </c>
       <c r="F44" s="2" t="n">
         <v>0</v>
@@ -5077,20 +5137,20 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
+          <t>SALDARRIAGA ECHEVERRIA BRYAN STEVEN</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
-        <v>-143.32</v>
+        <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0</v>
+        <v>219.81</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>218.16</v>
+        <v>0</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>0</v>
@@ -5104,23 +5164,23 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TORO BLACIO MARIA DEL CISNE</t>
+          <t>SOLANO DE LA SALA PAZ GONZALO PATRICIO</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>0</v>
+        <v>-143.32</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>406.22</v>
+        <v>0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>929.86</v>
+        <v>0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0</v>
+        <v>218.16</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -5131,39 +5191,66 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>TORO BLACIO MARIA DEL CISNE</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="2" t="n">
+        <v>406.22</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>929.86</v>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GUERRERO FAREZ FABIAN MAURICIO</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>WONG SANCHEZ PAULA SOFIA</t>
         </is>
       </c>
-      <c r="C47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="C48" s="5" t="n">
+      <c r="C48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49" s="5" t="n">
         <v>85092.72</v>
       </c>
-      <c r="D48" s="5" t="n">
+      <c r="D49" s="5" t="n">
         <v>51483.74</v>
       </c>
-      <c r="E48" s="5" t="n">
+      <c r="E49" s="5" t="n">
         <v>90445.31999999999</v>
       </c>
-      <c r="F48" s="5" t="n">
-        <v>33872.84</v>
-      </c>
-      <c r="G48" s="5" t="n">
+      <c r="F49" s="5" t="n">
+        <v>33898.26</v>
+      </c>
+      <c r="G49" s="5" t="n">
         <v>76987</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 17:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>3704.42</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>10 de 53</t>
+          <t>11 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
@@ -4199,7 +4199,7 @@
         <v>-94</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>2731.67</v>
+        <v>6436.09</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>38496.73</v>
+        <v>42201.15</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>14618.2</v>
+        <v>18322.62</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>58069.81</v>
+        <v>54365.39</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.201108821110937</v>
+        <v>0.2520721092790957</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>38496.73000000001</v>
+        <v>42201.15000000001</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>51643.28</v>
+        <v>47938.86</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4270770549060291</v>
+        <v>0.468173344999629</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-23 14:30:18
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -4577,7 +4577,7 @@
         <v>17.2</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>22.24</v>
+        <v>469.08</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>42201.15</v>
+        <v>42647.99</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5185,7 +5185,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>10758.81</v>
+        <v>11205.65</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-5226.809999999999</v>
+        <v>-5673.65</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1.944831887201735</v>
+        <v>2.025605567606652</v>
       </c>
     </row>
     <row r="5">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42201.15000000001</v>
+        <v>42647.99000000001</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>47938.86</v>
+        <v>47492.02</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.468173344999629</v>
+        <v>0.4731305221732282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-26 11:30:19
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1588,7 +1588,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>2146.66</v>
+        <v>2186.81</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -4307,7 +4307,7 @@
         <v>-40.75</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>2146.66</v>
+        <v>2186.81</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
@@ -4577,7 +4577,7 @@
         <v>17.2</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>469.08</v>
+        <v>558.45</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>42647.99</v>
+        <v>42777.51</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5185,7 +5185,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>11205.65</v>
+        <v>11295.02</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-5673.65</v>
+        <v>-5763.02</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2.025605567606652</v>
+        <v>2.041760665220535</v>
       </c>
     </row>
     <row r="5">
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>18322.62</v>
+        <v>18362.77</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>54365.39</v>
+        <v>54325.23999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2520721092790957</v>
+        <v>0.2526244699779235</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42647.99000000001</v>
+        <v>42777.51000000001</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>47492.02</v>
+        <v>47362.49999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4731305221732282</v>
+        <v>0.4745673979845355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-26 14:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -4577,7 +4577,7 @@
         <v>17.2</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>558.45</v>
+        <v>588.24</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>42777.51</v>
+        <v>42807.3</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5185,7 +5185,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>11295.02</v>
+        <v>11324.81</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-5763.02</v>
+        <v>-5792.809999999999</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2.041760665220535</v>
+        <v>2.047145697758496</v>
       </c>
     </row>
     <row r="5">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42777.51000000001</v>
+        <v>42807.3</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>47362.49999999999</v>
+        <v>47332.70999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4745673979845355</v>
+        <v>0.4748978838586773</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-27 15:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1288,7 +1288,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3704.42</v>
+        <v>3744.92</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -4199,7 +4199,7 @@
         <v>-94</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>6436.09</v>
+        <v>6476.59</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>42888.3</v>
+        <v>42928.8</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>18443.77</v>
+        <v>18484.27</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>54244.23999999999</v>
+        <v>54203.73999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2537388215745623</v>
+        <v>0.2542959973728817</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42888.3</v>
+        <v>42928.8</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>47251.70999999999</v>
+        <v>47211.20999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.475796485933383</v>
+        <v>0.4762457869707359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 14:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -2848,7 +2848,7 @@
         <v>0</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>5976.25</v>
+        <v>8664.85</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>0</v>
@@ -4577,7 +4577,7 @@
         <v>17.2</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>588.24</v>
+        <v>2985.34</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3000</v>
@@ -4847,7 +4847,7 @@
         <v>2928.27</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>5976.25</v>
+        <v>8664.85</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>2000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>48921.55</v>
+        <v>54007.25</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5284,13 +5284,13 @@
         <v>5532</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>11324.81</v>
+        <v>13721.91</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>-5792.809999999999</v>
+        <v>-8189.91</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2.047145697758496</v>
+        <v>2.480460954446855</v>
       </c>
     </row>
     <row r="5">
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>21555.61</v>
+        <v>24244.21</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>51132.39999999999</v>
+        <v>48443.8</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2965497335805451</v>
+        <v>0.3335379521326832</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>48962.05</v>
+        <v>54047.74999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>41177.95999999999</v>
+        <v>36092.26000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.543177774220349</v>
+        <v>0.5995977812738206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 08:30:17
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -802,7 +802,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>71.06</v>
+        <v>88.97</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>2304.79</v>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1942,13 +1942,13 @@
         <v>0</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>57.39</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>1863.61</v>
+        <v>1904.11</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0</v>
+        <v>154.56</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0</v>
+        <v>914.4</v>
       </c>
       <c r="O37" s="2" t="n">
         <v>0</v>
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>0</v>
+        <v>387.08</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>0</v>
@@ -3804,12 +3804,12 @@
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>1 de 53</t>
+          <t>2 de 53</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>9 de 53</t>
+          <t>10 de 53</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
@@ -3819,12 +3819,12 @@
       </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>17 de 53</t>
+          <t>19 de 53</t>
         </is>
       </c>
       <c r="N55" s="4" t="inlineStr">
         <is>
-          <t>2 de 53</t>
+          <t>3 de 53</t>
         </is>
       </c>
       <c r="O55" s="4" t="inlineStr">
@@ -3983,7 +3983,7 @@
         <v>11995.13</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2416.35</v>
+        <v>2434.26</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>6174</v>
@@ -4172,7 +4172,7 @@
         <v>1341.02</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>5678.57</v>
+        <v>5719.07</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>2500</v>
@@ -4469,7 +4469,7 @@
         <v>9608.059999999999</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1863.61</v>
+        <v>1961.5</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>4651</v>
@@ -4793,7 +4793,7 @@
         <v>0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0</v>
+        <v>1068.96</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>500</v>
@@ -4820,7 +4820,7 @@
         <v>0</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>0</v>
+        <v>387.08</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>0</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>54007.25</v>
+        <v>55619.59</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>218.16</v>
+        <v>372.72</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>-218.16</v>
+        <v>-372.72</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>0</v>
@@ -5452,13 +5452,13 @@
         <v>728</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>10403.84</v>
+        <v>10479.14</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-9675.84</v>
+        <v>-9751.139999999999</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14.29098901098901</v>
+        <v>14.39442307692308</v>
       </c>
     </row>
     <row r="12">
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>24244.21</v>
+        <v>24712.29</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>48443.8</v>
+        <v>47975.71999999999</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3335379521326832</v>
+        <v>0.3399775286185439</v>
       </c>
     </row>
     <row r="15">
@@ -5548,13 +5548,13 @@
         <v>402</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>596.34</v>
+        <v>1510.74</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>-194.34</v>
+        <v>-1108.74</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>1.483432835820896</v>
+        <v>3.758059701492537</v>
       </c>
     </row>
     <row r="16">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>54047.75</v>
+        <v>55660.09</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>36092.26000000001</v>
+        <v>34479.91999999999</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.5995977812738206</v>
+        <v>0.6174848438556862</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 14:30:16
</commit_message>
<xml_diff>
--- a/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
+++ b/data/GUERRERO FAREZ FABIAN MAURICIO.xlsx
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="2" t="n">
-        <v>1495.17</v>
+        <v>1472.52</v>
       </c>
       <c r="N23" s="2" t="n">
         <v>0</v>
@@ -4442,7 +4442,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1495.17</v>
+        <v>1472.52</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>3000</v>
@@ -5161,7 +5161,7 @@
         <v>90445.31999999999</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>55619.59</v>
+        <v>55596.94</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>76987</v>
@@ -5524,13 +5524,13 @@
         <v>72688.00999999999</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>24712.29</v>
+        <v>24689.64</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>47975.71999999999</v>
+        <v>47998.37</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3399775286185439</v>
+        <v>0.3396659228942985</v>
       </c>
     </row>
     <row r="15">
@@ -5567,13 +5567,13 @@
         <v>90140.00999999999</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55660.09</v>
+        <v>55637.44</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>34479.91999999999</v>
+        <v>34502.57000000001</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6174848438556862</v>
+        <v>0.6172335680903519</v>
       </c>
     </row>
   </sheetData>

</xml_diff>